<commit_message>
Correcion verdadera final borrar
</commit_message>
<xml_diff>
--- a/data/inputs/PruebaCorrecta.xlsx
+++ b/data/inputs/PruebaCorrecta.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/525260A030F8D24B/Documentos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DEB00A7-899A-464E-9CFD-3AFF7DA3FB30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4880A651-158C-492D-BCED-0426CDD81FBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3036" yWindow="3036" windowWidth="17280" windowHeight="8880" xr2:uid="{87EC7F06-7B0A-4F2E-8E12-705C7D6B230F}"/>
+    <workbookView xWindow="1116" yWindow="1116" windowWidth="17280" windowHeight="8880" xr2:uid="{87EC7F06-7B0A-4F2E-8E12-705C7D6B230F}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Boton descarga qr, correcion boton iniicar, cerrar sesion, permitir estar en inicio sin sesion
</commit_message>
<xml_diff>
--- a/data/inputs/PruebaCorrecta.xlsx
+++ b/data/inputs/PruebaCorrecta.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/525260A030F8D24B/Documentos/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/525260a030f8d24b/Documentos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4880A651-158C-492D-BCED-0426CDD81FBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{4880A651-158C-492D-BCED-0426CDD81FBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9C1C33B4-81C4-4ADC-A48E-B1CBD76F1FAF}"/>
   <bookViews>
-    <workbookView xWindow="1116" yWindow="1116" windowWidth="17280" windowHeight="8880" xr2:uid="{87EC7F06-7B0A-4F2E-8E12-705C7D6B230F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{87EC7F06-7B0A-4F2E-8E12-705C7D6B230F}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -193,10 +193,10 @@
     <t>Lactosa</t>
   </si>
   <si>
-    <t>Mostaza,Pescado</t>
-  </si>
-  <si>
     <t>Erase Una Vez</t>
+  </si>
+  <si>
+    <t>Mostaza, Pescado</t>
   </si>
 </sst>
 </file>
@@ -658,7 +658,7 @@
     </row>
     <row r="2" spans="1:7" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>20</v>
@@ -872,7 +872,7 @@
         <v>32</v>
       </c>
       <c r="F13" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">

</xml_diff>